<commit_message>
feat: cinematic Pillar Detail upgrade — presentation engine, command panel, exec brief
- Full 6-slide cinematic presentation mode (Focus Mode) with pillar-switching,
  animated SVG score ring, pillar-color accent lines on all financial tiles,
  and a new VER Asks slide (slide 6) wired to ver_asks data
- Cross-Pillar Command Panel (⚠ Command) with filterable open items across all pillars
- One-Click Exec Brief Generator (📄 Brief) with copyable email-ready summary
- Cinematic hero redesign: dark gradient, orb glow, faint grid, KPI strip, mini P&L bar
- Number key pillar navigation fixed inside presentation mode (no page reload)
- Intel Feed chip vertical alignment fix
- Typography scale-up across all presentation slides (54pt title, 108pt renewal days, etc.)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/VER_AnnualReview_Input_Form.xlsx
+++ b/assets/VER_AnnualReview_Input_Form.xlsx
@@ -1,58 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="READ ME FIRST" sheetId="1" r:id="rId1"/>
-    <sheet name="1. Header" sheetId="2" r:id="rId2"/>
-    <sheet name="2. Highlights" sheetId="3" r:id="rId3"/>
-    <sheet name="3. KPIs" sheetId="4" r:id="rId4"/>
-    <sheet name="4. Wins" sheetId="5" r:id="rId5"/>
-    <sheet name="5. Year Ahead" sheetId="6" r:id="rId6"/>
-    <sheet name="6. Custom Notes" sheetId="7" r:id="rId7"/>
+    <sheet name="READ ME FIRST" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="1. Header" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2. Highlights" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="3. KPIs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="4. Wins" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="5. Year Ahead" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="6. Custom Notes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -71,13 +48,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -402,294 +446,745 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>VER ANNUAL REVIEW INPUT FORM</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>VER ANNUAL REVIEW INPUT FORM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" t="str">
-        <v>INSTRUCTIONS</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>Fill in each tab with your meeting data.</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fill in each tab with your meeting data.</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>All fields are optional — fill what you have.</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>All fields are optional — fill what you have.</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>Return this file to VER or paste values into the generator.</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Return this file to VER or paste values into the generator.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>Field</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Review Title</v>
-      </c>
-      <c r="B2" t="str">
-        <v/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Review Title</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Salesforce DET — FY26 Vendor Engagement &amp; Reliability Annual Review</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>Period</v>
-      </c>
-      <c r="B3" t="str">
-        <v/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FY26 (Feb 2025 – Jan 2026)</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>Presenter</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Presenter</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Casey Candelaria, VER Intelligence Lead</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>Audience</v>
-      </c>
-      <c r="B5" t="str">
-        <v/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Audience</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Joe Martinez (Org President), Roger Espinoza (DA&amp;O Director), DET Leadership</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B6" t="str">
-        <v/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>N/A — Portfolio-Level Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FY</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>Category</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Highlight</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Impact</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Highlight</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$8.3M in negotiated rate reductions across 12 preferred suppliers</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>$8.3M below FY26 benchmark baseline — 5.6% blended rate improvement</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>47 CQBRs delivered — 100% of Tier 1 suppliers reviewed on schedule</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>First year full CQBR coverage achieved across all Tier 1 vendors</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Risk Mitigation</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3 high-risk suppliers identified and remediated before escalation</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cognizant, NTT Data, and IBM all recovered to Green within quarter</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>94% SLA compliance rate across portfolio — up from 89% in FY25</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>5-point improvement; attributed to CQBR accountability cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>VER Intelligence Hub deployed — first AI-enabled vendor intelligence platform in DET</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hub now used by 23 stakeholders; CQBR generation time reduced from 3 days to 4 hours</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>KPI</v>
-      </c>
-      <c r="B1" t="str">
-        <v>FY Target</v>
-      </c>
-      <c r="C1" t="str">
-        <v>FY Actual</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Status</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>FY Target</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>FY Actual</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Portfolio Spend vs Budget</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$148M</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>$142M</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SLA Compliance Rate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CQBR On-Time Delivery</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Preferred Supplier Rate vs Benchmark</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>-5.6%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Open Governance Items at Year End</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vendor Satisfaction (VER Survey)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7.5/10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>8.1/10</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>#</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Win</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Impact</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$8.3M savings from rate renegotiations</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Exceeded $6M FY26 savings target by 38%</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <v/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>First full CQBR cycle — all Tier 1 vendors reviewed on schedule</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>47 CQBRs delivered; institutional memory now captured for every supplier</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>VER Intelligence Hub launched and adopted by leadership</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Joe Martinez formally endorsed hub for broader org packaging</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Three high-risk vendor relationships recovered to Green without escalation</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cognizant KT, NTT Data SLA, IBM renewal all resolved within quarter</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>94% portfolio SLA compliance — 5-point gain from FY25</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Best compliance rate since DET began tracking in FY23</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>Initiative</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Goal</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Target Date</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Initiative</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Goal</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Target Date</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CQBR Automation Expansion</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Reduce generator cycle time from 4 hours to 30 minutes with pre-loaded templates</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>VER Team</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tier 3 Vendor Rationalization</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Identify 15 vendors for consolidation or exit — target $4M additional savings</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>VER Analyst</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Stakeholder Survey v2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Expand survey to all 16 Tier 1 vendors — quarterly cadence automated</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>VER Team</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>VER Hub Packaging</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Package hub for broader Salesforce org adoption — Joe office hours presentation complete</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Casey Candelaria</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rate Benchmark Refresh</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Refresh all 16 Tier 1 rate benchmarks using current market data</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>VER Intelligence</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>Label</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Notes</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FY27 Priority</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Tier 3 rationalization is the single highest-value FY27 initiative — estimated $3-5M savings if 8 vendors consolidated or exited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Recognition</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Alex Rivera recognized for building the CQBR generator and rate benchmark engine from scratch. Debs Garcia recognized for 47 on-time CQBR completions with zero misses.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>